<commit_message>
docs(javni-sajt): usklađeni statusi slika — sistemi bez šifre, SATA kandidati, ponuda nepotvrđena
- AGILIS X-TREME i ONYX HD TROPICAL: bez zahteva za fotografijom jedne ambalaže, odluka o prikazu sistema
- 7 SATA slika srodnih artikala: kandidati, bez uvoza dok se ne potvrdi šta prikazuju
- fotografija ambalaže traži se samo ako je artikal u ponudi; ništa se ne uklanja
Statusi su isti u glavnom (privatnom) Excelu, javnoj kopiji i magacinskoj tabeli.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/javni-sajt/SLIKE_ZA_PRONALAZENJE.xlsx
+++ b/docs/javni-sajt/SLIKE_ZA_PRONALAZENJE.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -526,190 +526,236 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Pregled sa slikama</t>
+          <t>Ponuda i magacin</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>~/Carsystem/radno/slike-za-pronalazenje/PREGLED_SPORNIH_SLIKA.html (i .jpg): 8 Cosmos sa zajedničkom slikom, 7 SATA sa slikom srodnog artikla, FO-314; neslaganje 175/185 ml za Chrome 450 / Gold 451 je istaknuto — katalog NIJE menjan.</t>
+          <t>Za 25 proizvoda bez pronađene slike ponuda nije potvrđena; odsustvo iz pregledanog šifarnika NE znači uklanjanje sa sajta. Trenutno stanje magacina je nepoznato dok ga vlasnik ne proveri (spisak: MAGACIN_PROVERA.xlsx, privatno).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr"/>
-      <c r="B8" s="2" t="n"/>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Sistemi bez šifre</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>AGILIS X-TREME i ONYX HD TROPICAL: nema zahteva za fotografiju jedne ambalaže — traži se odluka o prikazu sistema.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Stanje</t>
+          <t>SATA — slike srodnih artikala</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Broj</t>
+          <t>7 slika su samo kandidati: ne uvoze se dok se ne potvrdi šta tačno prikazuju (i dok nema prava).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>136</v>
+          <t>Pregled sa slikama</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>~/Carsystem/radno/slike-za-pronalazenje/PREGLED_SPORNIH_SLIKA.html (i .jpg): 8 Cosmos sa zajedničkom slikom, 7 SATA sa slikom srodnog artikla, FO-314; neslaganje 175/185 ml za Chrome 450 / Gold 451 je istaknuto — katalog NIJE menjan.</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>23</v>
-      </c>
+      <c r="A11" s="1" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>nije pronađeno — placeholder prihvaćen</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>12</v>
+          <t>Stanje</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Broj</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i Vašu odluku o zajedničkoj slici</t>
+          <t>pronađeno — čeka pravo</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>8</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>čeka potvrdu identiteta</t>
+          <t>nije pronađeno — placeholder prihvaćen</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr"/>
-      <c r="B16" s="2" t="n"/>
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>pronađeno — čeka pravo i Vašu odluku o zajedničkoj slici</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Po brendu</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Stanja</t>
-        </is>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>R-M</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>nije pronađeno — potrebna Vaša fotografija: 15; čeka potvrdu identiteta: 1; pronađeno — čeka pravo: 1</t>
-        </is>
+          <t>čeka potvrdu identiteta</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>baslac</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>čeka potvrdu identiteta: 1; nije pronađeno — potrebna Vaša fotografija: 3</t>
-        </is>
+          <t>nije pronađeno — čeka odluku o prikazu sistema</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Norbin</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>nije pronađeno — potrebna Vaša fotografija: 4</t>
-        </is>
-      </c>
+      <c r="A20" s="1" t="inlineStr"/>
+      <c r="B20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Cosmos Lac</t>
+          <t>Po brendu</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i Vašu odluku o zajedničkoj slici: 8; pronađeno — čeka pravo: 2; čeka potvrdu identiteta: 1</t>
+          <t>Stanja</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>SATA</t>
+          <t>R-M</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo: 133; nije pronađeno — placeholder prihvaćen: 12; pronađeno — čeka pravo i potvrdu varijante: 7; nije pronađeno — potrebna Vaša fotografija: 1</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi): 13; nije pronađeno — čeka odluku o prikazu sistema: 2; čeka potvrdu identiteta: 1; pronađeno — čeka pravo: 1</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr"/>
-      <c r="B23" s="2" t="n"/>
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>baslac</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>čeka potvrdu identiteta: 1; nije pronađeno — potrebna Vaša fotografija (ako je u ponudi): 3</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Gde su fajlovi</t>
+          <t>Norbin</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>~/Carsystem/radno/slike-za-pronalazenje/preuzeto/&lt;brend&gt;/ — van git-a, nije objavljeno. SATA _manifest.json ima URL, SHA-256 i stranicu artikla za svaki fajl.</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi): 4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
+          <t>Cosmos Lac</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>pronađeno — čeka pravo i Vašu odluku o zajedničkoj slici: 8; pronađeno — čeka pravo: 2; čeka potvrdu identiteta: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>SATA</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>pronađeno — čeka pravo: 133; nije pronađeno — placeholder prihvaćen: 12; kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo: 7; nije pronađeno — potrebna Vaša fotografija (ako je u ponudi): 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr"/>
+      <c r="B27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Gde su fajlovi</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>~/Carsystem/radno/slike-za-pronalazenje/preuzeto/&lt;brend&gt;/ — van git-a, nije objavljeno. SATA _manifest.json ima URL, SHA-256 i stranicu artikla za svaki fajl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
           <t>Pravila</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Podudaranje „Potvrđeno” samo kad slika nosi tačnu šifru/naziv ili je sopstvena glavna slika artikla na stranici proizvođača. Zajednička slika porodice je označena posebno. Šifre se ne izmišljaju.</t>
         </is>
@@ -893,7 +939,7 @@
       <c r="M2" s="2" t="inlineStr"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -910,7 +956,7 @@
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -956,7 +1002,7 @@
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Odluka o prikazu SISTEMA AGILIS X-TREME (nema jednu ambalažu): npr. bez fotografije, zvanična slika sistema/kolekcije ili konkretna komponenta — NE fotografisati jednu limenku</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -973,7 +1019,7 @@
       <c r="R3" s="5" t="inlineStr"/>
       <c r="S3" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — čeka odluku o prikazu sistema</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1136,7 @@
       <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -1107,7 +1153,7 @@
       <c r="R5" s="5" t="inlineStr"/>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1203,7 @@
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -1174,7 +1220,7 @@
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1361,7 @@
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
@@ -1332,7 +1378,7 @@
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1428,7 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
@@ -1399,7 +1445,7 @@
       <c r="R9" s="5" t="inlineStr"/>
       <c r="S9" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1495,7 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
@@ -1466,7 +1512,7 @@
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1516,7 +1562,7 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
@@ -1533,7 +1579,7 @@
       <c r="R11" s="5" t="inlineStr"/>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1629,7 @@
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
@@ -1600,7 +1646,7 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1696,7 @@
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1667,7 +1713,7 @@
       <c r="R13" s="5" t="inlineStr"/>
       <c r="S13" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1759,7 @@
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Odluka o prikazu SISTEMA ONYX HD TROPICAL (nema jednu ambalažu): npr. bez fotografije, zvanična slika sistema/kolekcije ili konkretna komponenta — NE fotografisati jednu limenku</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
@@ -1730,7 +1776,7 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — čeka odluku o prikazu sistema</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1826,7 @@
       <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1797,7 +1843,7 @@
       <c r="R15" s="5" t="inlineStr"/>
       <c r="S15" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1893,7 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
@@ -1864,7 +1910,7 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1960,7 @@
       <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
@@ -1931,7 +1977,7 @@
       <c r="R17" s="5" t="inlineStr"/>
       <c r="S17" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -1981,7 +2027,7 @@
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
@@ -1998,7 +2044,7 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2157,7 @@
       <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
@@ -2128,7 +2174,7 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2224,7 @@
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
@@ -2195,7 +2241,7 @@
       <c r="R21" s="5" t="inlineStr"/>
       <c r="S21" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2291,7 @@
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
@@ -2262,7 +2308,7 @@
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2362,7 @@
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
@@ -2333,7 +2379,7 @@
       <c r="R23" s="5" t="inlineStr"/>
       <c r="S23" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -2387,7 +2433,7 @@
       <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
@@ -2404,7 +2450,7 @@
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2504,7 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O25" s="2" t="inlineStr">
@@ -2475,7 +2521,7 @@
       <c r="R25" s="5" t="inlineStr"/>
       <c r="S25" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2575,7 @@
       <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Vaša fotografija ambalaže (proizvođač ne objavljuje sliku ove šifre)</t>
+          <t>Vaša fotografija ambalaže, ako je artikal u našoj ponudi (proizvođač ne objavljuje sliku ove šifre)</t>
         </is>
       </c>
       <c r="O26" s="2" t="inlineStr">
@@ -2546,7 +2592,7 @@
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6814,7 @@
       </c>
       <c r="S72" s="5" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
         </is>
       </c>
     </row>
@@ -8078,7 +8124,7 @@
       </c>
       <c r="S86" s="5" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
         </is>
       </c>
     </row>
@@ -8173,7 +8219,7 @@
       </c>
       <c r="S87" s="5" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
         </is>
       </c>
     </row>
@@ -9883,7 +9929,7 @@
       </c>
       <c r="S105" s="5" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
         </is>
       </c>
     </row>
@@ -10738,7 +10784,7 @@
       </c>
       <c r="S114" s="5" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10879,7 @@
       </c>
       <c r="S115" s="5" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
         </is>
       </c>
     </row>
@@ -11573,7 +11619,7 @@
       <c r="R123" s="5" t="inlineStr"/>
       <c r="S123" s="5" t="inlineStr">
         <is>
-          <t>nije pronađeno — potrebna Vaša fotografija</t>
+          <t>nije pronađeno — potrebna Vaša fotografija (ako je u ponudi)</t>
         </is>
       </c>
     </row>
@@ -13868,7 +13914,7 @@
       </c>
       <c r="S148" s="5" t="inlineStr">
         <is>
-          <t>pronađeno — čeka pravo i potvrdu varijante</t>
+          <t>kandidat (slika srodnog artikla) — bez uvoza dok se ne potvrdi šta prikazuje; čeka i pravo</t>
         </is>
       </c>
     </row>

</xml_diff>